<commit_message>
Update platform URL to pro-palenke-vw-two.vercel.app.
Keep docs, final formats, and generate scripts pointing at the current validation deployment.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/final-formats/02_Matriz_cumplimiento_ANGEL_MATEUS_final.xlsx
+++ b/docs/final-formats/02_Matriz_cumplimiento_ANGEL_MATEUS_final.xlsx
@@ -1197,7 +1197,7 @@
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs ; informes ABRIL/MAYO 2026</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs ; informes ABRIL/MAYO 2026</t>
         </is>
       </c>
       <c r="H9" s="12" t="inlineStr">
@@ -1238,12 +1238,12 @@
       </c>
       <c r="F10" s="12" t="inlineStr">
         <is>
-          <t>MVP funcional. Catálogo de módulos/URLs: https://dev-palenke-two.vercel.app/docs/modulos-y-urls. Docs generales: https://dev-palenke-two.vercel.app/docs.</t>
+          <t>MVP funcional. Catálogo de módulos/URLs: https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls. Docs generales: https://pro-palenke-vw-two.vercel.app/docs.</t>
         </is>
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/ ; https://dev-palenke-two.vercel.app/docs/modulos-y-urls ; https://dev-palenke-two.vercel.app/docs</t>
+          <t>https://pro-palenke-vw-two.vercel.app/ ; https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls ; https://pro-palenke-vw-two.vercel.app/docs</t>
         </is>
       </c>
       <c r="H10" s="12" t="inlineStr">
@@ -1284,12 +1284,12 @@
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>Sistema de usuarios y roles operativo. Guía legible: https://dev-palenke-two.vercel.app/docs/accesos. Login https://dev-palenke-two.vercel.app/login. Admin angelarrieta34@gmail.com / welcome123. Interno fconu@renacientes.org / @welcome123. Panel https://dev-palenke-two.vercel.app/admin.</t>
+          <t>Sistema de usuarios y roles operativo. Guía legible: https://pro-palenke-vw-two.vercel.app/docs/accesos. Login https://pro-palenke-vw-two.vercel.app/login. Admin angelarrieta34@gmail.com / welcome123. Interno fconu@renacientes.org / @welcome123. Panel https://pro-palenke-vw-two.vercel.app/admin.</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/accesos ; https://dev-palenke-two.vercel.app/login ; https://dev-palenke-two.vercel.app/admin</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/accesos ; https://pro-palenke-vw-two.vercel.app/login ; https://pro-palenke-vw-two.vercel.app/admin</t>
         </is>
       </c>
       <c r="H11" s="12" t="inlineStr">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="G12" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/modulos-y-urls ; https://dev-palenke-two.vercel.app/gobierno-propio ; https://dev-palenke-two.vercel.app/biblioteca ; https://dev-palenke-two.vercel.app/memoria-afroterritorial</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls ; https://pro-palenke-vw-two.vercel.app/gobierno-propio ; https://pro-palenke-vw-two.vercel.app/biblioteca ; https://pro-palenke-vw-two.vercel.app/memoria-afroterritorial</t>
         </is>
       </c>
       <c r="H12" s="12" t="inlineStr">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/modulos-y-urls ; https://dev-palenke-two.vercel.app/biblioteca ; https://dev-palenke-two.vercel.app/memoria-afroterritorial ; https://dev-palenke-two.vercel.app/memoria-afroterritorial/mediateca-ubuntu</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls ; https://pro-palenke-vw-two.vercel.app/biblioteca ; https://pro-palenke-vw-two.vercel.app/memoria-afroterritorial ; https://pro-palenke-vw-two.vercel.app/memoria-afroterritorial/mediateca-ubuntu</t>
         </is>
       </c>
       <c r="H13" s="12" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="G14" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/modulos-y-urls ; https://dev-palenke-two.vercel.app/mujeres-juventudes-ninez</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls ; https://pro-palenke-vw-two.vercel.app/mujeres-juventudes-ninez</t>
         </is>
       </c>
       <c r="H14" s="12" t="inlineStr">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/modulos-y-urls ; https://dev-palenke-two.vercel.app/estadisticas ; https://dev-palenke-two.vercel.app/scita ; https://dev-palenke-two.vercel.app/admin/dashboards ; Geoportal siguiente etapa: https://dev-palenke-two.vercel.app/geoportal</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls ; https://pro-palenke-vw-two.vercel.app/estadisticas ; https://pro-palenke-vw-two.vercel.app/scita ; https://pro-palenke-vw-two.vercel.app/admin/dashboards ; Geoportal siguiente etapa: https://pro-palenke-vw-two.vercel.app/geoportal</t>
         </is>
       </c>
       <c r="H15" s="12" t="inlineStr">
@@ -1514,12 +1514,12 @@
       </c>
       <c r="F16" s="12" t="inlineStr">
         <is>
-          <t>Seguridad básica operativa (HTTPS + sesión/roles). Entrada admin/interno vía https://dev-palenke-two.vercel.app/login ; credenciales admin e internas en https://dev-palenke-two.vercel.app/docs/accesos</t>
+          <t>Seguridad básica operativa (HTTPS + sesión/roles). Entrada admin/interno vía https://pro-palenke-vw-two.vercel.app/login ; credenciales admin e internas en https://pro-palenke-vw-two.vercel.app/docs/accesos</t>
         </is>
       </c>
       <c r="G16" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/accesos ; https://dev-palenke-two.vercel.app/login ; https://dev-palenke-two.vercel.app/admin</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/accesos ; https://pro-palenke-vw-two.vercel.app/login ; https://pro-palenke-vw-two.vercel.app/admin</t>
         </is>
       </c>
       <c r="H16" s="12" t="inlineStr">
@@ -1560,12 +1560,12 @@
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>Código en GitHub privado + guía https://dev-palenke-two.vercel.app/docs/repositorio-codigo. Accesos plataforma: https://dev-palenke-two.vercel.app/docs/accesos. Pendiente acta formal de transferencia.</t>
+          <t>Código en GitHub privado + guía https://pro-palenke-vw-two.vercel.app/docs/repositorio-codigo. Accesos plataforma: https://pro-palenke-vw-two.vercel.app/docs/accesos. Pendiente acta formal de transferencia.</t>
         </is>
       </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/repositorio-codigo ; https://github.com/anuidev8/palenke (privado; invitar por email) ; https://dev-palenke-two.vercel.app/docs/accesos</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/repositorio-codigo ; https://github.com/anuidev8/palenke (privado; invitar por email) ; https://pro-palenke-vw-two.vercel.app/docs/accesos</t>
         </is>
       </c>
       <c r="H17" s="12" t="inlineStr">
@@ -1606,12 +1606,12 @@
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>Documentación técnica legible en https://dev-palenke-two.vercel.app/docs (arquitectura/DB: https://dev-palenke-two.vercel.app/docs/arquitectura-y-base-de-datos; construcción por módulo: https://dev-palenke-two.vercel.app/docs/como-esta-construido) y paquete docs/technical en el repositorio.</t>
+          <t>Documentación técnica legible en https://pro-palenke-vw-two.vercel.app/docs (arquitectura/DB: https://pro-palenke-vw-two.vercel.app/docs/arquitectura-y-base-de-datos; construcción por módulo: https://pro-palenke-vw-two.vercel.app/docs/como-esta-construido) y paquete docs/technical en el repositorio.</t>
         </is>
       </c>
       <c r="G18" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs ; https://dev-palenke-two.vercel.app/docs/arquitectura-y-base-de-datos ; https://dev-palenke-two.vercel.app/docs/como-esta-construido ; docs/technical/palenke-mvp-technical-documentation.md</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs ; https://pro-palenke-vw-two.vercel.app/docs/arquitectura-y-base-de-datos ; https://pro-palenke-vw-two.vercel.app/docs/como-esta-construido ; docs/technical/palenke-mvp-technical-documentation.md</t>
         </is>
       </c>
       <c r="H18" s="12" t="inlineStr">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="G19" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs</t>
         </is>
       </c>
       <c r="H19" s="12" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="G20" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/modulos-y-urls ; https://dev-palenke-two.vercel.app/ ; https://github.com/anuidev8/palenke</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls ; https://pro-palenke-vw-two.vercel.app/ ; https://github.com/anuidev8/palenke</t>
         </is>
       </c>
       <c r="H20" s="12" t="inlineStr">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="G21" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/modulos-y-urls ; https://dev-palenke-two.vercel.app/</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls ; https://pro-palenke-vw-two.vercel.app/</t>
         </is>
       </c>
       <c r="H21" s="12" t="inlineStr">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="G22" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/accesos ; https://dev-palenke-two.vercel.app/login ; https://dev-palenke-two.vercel.app/admin</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/accesos ; https://pro-palenke-vw-two.vercel.app/login ; https://pro-palenke-vw-two.vercel.app/admin</t>
         </is>
       </c>
       <c r="H22" s="12" t="inlineStr">
@@ -1841,7 +1841,7 @@
       </c>
       <c r="G23" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/modulos-y-urls ; https://dev-palenke-two.vercel.app/gobierno-propio ; https://dev-palenke-two.vercel.app/biblioteca</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls ; https://pro-palenke-vw-two.vercel.app/gobierno-propio ; https://pro-palenke-vw-two.vercel.app/biblioteca</t>
         </is>
       </c>
       <c r="H23" s="12" t="inlineStr">
@@ -1887,7 +1887,7 @@
       </c>
       <c r="G24" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/modulos-y-urls ; https://dev-palenke-two.vercel.app/biblioteca ; https://dev-palenke-two.vercel.app/memoria-afroterritorial</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls ; https://pro-palenke-vw-two.vercel.app/biblioteca ; https://pro-palenke-vw-two.vercel.app/memoria-afroterritorial</t>
         </is>
       </c>
       <c r="H24" s="12" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="G25" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/modulos-y-urls ; https://dev-palenke-two.vercel.app/mujeres-juventudes-ninez</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls ; https://pro-palenke-vw-two.vercel.app/mujeres-juventudes-ninez</t>
         </is>
       </c>
       <c r="H25" s="12" t="inlineStr">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="G26" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/modulos-y-urls ; https://dev-palenke-two.vercel.app/estadisticas ; https://dev-palenke-two.vercel.app/scita ; https://dev-palenke-two.vercel.app/admin/dashboards</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls ; https://pro-palenke-vw-two.vercel.app/estadisticas ; https://pro-palenke-vw-two.vercel.app/scita ; https://pro-palenke-vw-two.vercel.app/admin/dashboards</t>
         </is>
       </c>
       <c r="H26" s="12" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="G27" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/modulos-y-urls ; https://dev-palenke-two.vercel.app/geoportal ; https://dev-palenke-two.vercel.app/docs/accesos (siguiente etapa / no MVP)</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls ; https://pro-palenke-vw-two.vercel.app/geoportal ; https://pro-palenke-vw-two.vercel.app/docs/accesos (siguiente etapa / no MVP)</t>
         </is>
       </c>
       <c r="H27" s="12" t="inlineStr">
@@ -2071,7 +2071,7 @@
       </c>
       <c r="G28" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/accesos ; https://dev-palenke-two.vercel.app/login ; https://dev-palenke-two.vercel.app/admin</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/accesos ; https://pro-palenke-vw-two.vercel.app/login ; https://pro-palenke-vw-two.vercel.app/admin</t>
         </is>
       </c>
       <c r="H28" s="12" t="inlineStr">
@@ -2117,7 +2117,7 @@
       </c>
       <c r="G29" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/repositorio-codigo ; https://github.com/anuidev8/palenke</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/repositorio-codigo ; https://github.com/anuidev8/palenke</t>
         </is>
       </c>
       <c r="H29" s="12" t="inlineStr">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="G30" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs ; https://dev-palenke-two.vercel.app/docs/arquitectura-y-base-de-datos ; https://dev-palenke-two.vercel.app/docs/como-esta-construido</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs ; https://pro-palenke-vw-two.vercel.app/docs/arquitectura-y-base-de-datos ; https://pro-palenke-vw-two.vercel.app/docs/como-esta-construido</t>
         </is>
       </c>
       <c r="H30" s="12" t="inlineStr">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="G31" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/arquitectura-y-base-de-datos ; https://dev-palenke-two.vercel.app/gobierno-propio ; https://dev-palenke-two.vercel.app/biblioteca</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/arquitectura-y-base-de-datos ; https://pro-palenke-vw-two.vercel.app/gobierno-propio ; https://pro-palenke-vw-two.vercel.app/biblioteca</t>
         </is>
       </c>
       <c r="H31" s="12" t="inlineStr">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="G32" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/modulos-y-urls ; https://dev-palenke-two.vercel.app/biblioteca</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls ; https://pro-palenke-vw-two.vercel.app/biblioteca</t>
         </is>
       </c>
       <c r="H32" s="12" t="inlineStr">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="G33" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/modulos-y-urls ; https://dev-palenke-two.vercel.app/gobierno-propio ; https://dev-palenke-two.vercel.app/admin/accs ; https://dev-palenke-two.vercel.app/docs/accesos</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls ; https://pro-palenke-vw-two.vercel.app/gobierno-propio ; https://pro-palenke-vw-two.vercel.app/admin/accs ; https://pro-palenke-vw-two.vercel.app/docs/accesos</t>
         </is>
       </c>
       <c r="H33" s="12" t="inlineStr">
@@ -2347,7 +2347,7 @@
       </c>
       <c r="G34" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/modulos-y-urls ; https://dev-palenke-two.vercel.app/incidencia ; https://dev-palenke-two.vercel.app/noticias</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls ; https://pro-palenke-vw-two.vercel.app/incidencia ; https://pro-palenke-vw-two.vercel.app/noticias</t>
         </is>
       </c>
       <c r="H34" s="12" t="inlineStr">
@@ -2393,7 +2393,7 @@
       </c>
       <c r="G35" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/arquitectura-y-base-de-datos ; https://dev-palenke-two.vercel.app/docs ; https://dev-palenke-two.vercel.app/</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/arquitectura-y-base-de-datos ; https://pro-palenke-vw-two.vercel.app/docs ; https://pro-palenke-vw-two.vercel.app/</t>
         </is>
       </c>
       <c r="H35" s="12" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="G36" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs</t>
         </is>
       </c>
       <c r="H36" s="12" t="inlineStr">
@@ -2485,7 +2485,7 @@
       </c>
       <c r="G37" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs ; https://dev-palenke-two.vercel.app/docs/arquitectura-y-base-de-datos ; https://dev-palenke-two.vercel.app/docs/como-esta-construido</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs ; https://pro-palenke-vw-two.vercel.app/docs/arquitectura-y-base-de-datos ; https://pro-palenke-vw-two.vercel.app/docs/como-esta-construido</t>
         </is>
       </c>
       <c r="H37" s="12" t="inlineStr">
@@ -2531,7 +2531,7 @@
       </c>
       <c r="G38" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs</t>
         </is>
       </c>
       <c r="H38" s="12" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="G39" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/modulos-y-urls ; https://dev-palenke-two.vercel.app/ ; https://dev-palenke-two.vercel.app/docs/repositorio-codigo</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls ; https://pro-palenke-vw-two.vercel.app/ ; https://pro-palenke-vw-two.vercel.app/docs/repositorio-codigo</t>
         </is>
       </c>
       <c r="H39" s="12" t="inlineStr">
@@ -2623,7 +2623,7 @@
       </c>
       <c r="G40" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/arquitectura-y-base-de-datos ; https://dev-palenke-two.vercel.app/gobierno-propio ; https://dev-palenke-two.vercel.app/biblioteca</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/arquitectura-y-base-de-datos ; https://pro-palenke-vw-two.vercel.app/gobierno-propio ; https://pro-palenke-vw-two.vercel.app/biblioteca</t>
         </is>
       </c>
       <c r="H40" s="12" t="inlineStr">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="G41" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/modulos-y-urls ; https://dev-palenke-two.vercel.app/biblioteca</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls ; https://pro-palenke-vw-two.vercel.app/biblioteca</t>
         </is>
       </c>
       <c r="H41" s="12" t="inlineStr">
@@ -2715,7 +2715,7 @@
       </c>
       <c r="G42" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/modulos-y-urls ; https://dev-palenke-two.vercel.app/gobierno-propio ; https://dev-palenke-two.vercel.app/admin/accs</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls ; https://pro-palenke-vw-two.vercel.app/gobierno-propio ; https://pro-palenke-vw-two.vercel.app/admin/accs</t>
         </is>
       </c>
       <c r="H42" s="12" t="inlineStr">
@@ -2761,7 +2761,7 @@
       </c>
       <c r="G43" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/modulos-y-urls ; https://dev-palenke-two.vercel.app/incidencia</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls ; https://pro-palenke-vw-two.vercel.app/incidencia</t>
         </is>
       </c>
       <c r="H43" s="12" t="inlineStr">
@@ -2807,7 +2807,7 @@
       </c>
       <c r="G44" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/arquitectura-y-base-de-datos ; https://dev-palenke-two.vercel.app/</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/arquitectura-y-base-de-datos ; https://pro-palenke-vw-two.vercel.app/</t>
         </is>
       </c>
       <c r="H44" s="12" t="inlineStr">
@@ -2853,7 +2853,7 @@
       </c>
       <c r="G45" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs</t>
         </is>
       </c>
       <c r="H45" s="12" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="G46" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs ; https://dev-palenke-two.vercel.app/docs/arquitectura-y-base-de-datos ; https://dev-palenke-two.vercel.app/docs/como-esta-construido</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs ; https://pro-palenke-vw-two.vercel.app/docs/arquitectura-y-base-de-datos ; https://pro-palenke-vw-two.vercel.app/docs/como-esta-construido</t>
         </is>
       </c>
       <c r="H46" s="12" t="inlineStr">
@@ -2945,7 +2945,7 @@
       </c>
       <c r="G47" s="12" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs</t>
         </is>
       </c>
       <c r="H47" s="12" t="inlineStr">
@@ -3172,7 +3172,7 @@
       </c>
       <c r="E7" s="1" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs ; https://dev-palenke-two.vercel.app/docs/informe-y-matriz ; https://dev-palenke-two.vercel.app/docs/modulos-y-urls ; https://dev-palenke-two.vercel.app/docs/como-esta-construido</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs ; https://pro-palenke-vw-two.vercel.app/docs/informe-y-matriz ; https://pro-palenke-vw-two.vercel.app/docs/modulos-y-urls ; https://pro-palenke-vw-two.vercel.app/docs/como-esta-construido</t>
         </is>
       </c>
       <c r="F7" s="1" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="E13" s="1" t="inlineStr">
         <is>
-          <t>https://dev-palenke-two.vercel.app/docs/repositorio-codigo ; https://dev-palenke-two.vercel.app/docs/accesos ; https://dev-palenke-two.vercel.app/docs/arquitectura-y-base-de-datos ; https://dev-palenke-two.vercel.app/docs/como-esta-construido ; https://github.com/anuidev8/palenke</t>
+          <t>https://pro-palenke-vw-two.vercel.app/docs/repositorio-codigo ; https://pro-palenke-vw-two.vercel.app/docs/accesos ; https://pro-palenke-vw-two.vercel.app/docs/arquitectura-y-base-de-datos ; https://pro-palenke-vw-two.vercel.app/docs/como-esta-construido ; https://github.com/anuidev8/palenke</t>
         </is>
       </c>
       <c r="F13" s="1" t="inlineStr">

</xml_diff>